<commit_message>
Auto-refresh chess stats 2026-09-06
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>89 (53.0%)</t>
+          <t>90 (52.9%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (3.0%)</t>
+          <t>5 (2.9%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>74 (44.0%)</t>
+          <t>75 (44.1%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>43 (47.8%)</t>
+          <t>44 (47.3%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (5.6%)</t>
+          <t>5 (5.4%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>42 (46.7%)</t>
+          <t>44 (47.3%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>25 (48.1%)</t>
+          <t>26 (49.1%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>26 (50.0%)</t>
+          <t>26 (49.1%)</t>
         </is>
       </c>
     </row>
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17 (65.4%)</t>
+          <t>18 (66.7%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (3.8%)</t>
+          <t>1 (3.7%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8 (30.8%)</t>
+          <t>8 (29.6%)</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -755,24 +755,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>12 (63.2%)</t>
+          <t>7 (36.8%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1 (5.3%)</t>
+          <t>2 (10.5%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6 (31.6%)</t>
+          <t>10 (52.6%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -780,42 +780,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8 (42.1%)</t>
+          <t>12 (63.2%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.3%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11 (57.9%)</t>
+          <t>6 (31.6%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>7 (38.9%)</t>
+          <t>8 (42.1%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2 (11.1%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>9 (50.0%)</t>
+          <t>11 (57.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-07
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>90 (52.9%)</t>
+          <t>91 (52.6%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>75 (44.1%)</t>
+          <t>77 (44.5%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>44 (47.3%)</t>
+          <t>46 (47.9%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (5.4%)</t>
+          <t>6 (6.2%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44 (47.3%)</t>
+          <t>44 (45.8%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>31 (57.4%)</t>
+          <t>32 (58.2%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (1.9%)</t>
+          <t>1 (1.8%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>22 (40.7%)</t>
+          <t>22 (40.0%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12 (41.4%)</t>
+          <t>12 (40.0%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (6.9%)</t>
+          <t>2 (6.7%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15 (51.7%)</t>
+          <t>16 (53.3%)</t>
         </is>
       </c>
     </row>
@@ -726,11 +726,11 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11 (52.4%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-08
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>91 (52.6%)</t>
+          <t>91 (52.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>77 (44.5%)</t>
+          <t>79 (45.1%)</t>
         </is>
       </c>
     </row>
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>46 (47.9%)</t>
+          <t>46 (47.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>44 (45.8%)</t>
+          <t>45 (46.4%)</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -655,42 +655,42 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12 (48.0%)</t>
+          <t>11 (44.0%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>12 (48.0%)</t>
+          <t>14 (56.0%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10 (41.7%)</t>
+          <t>12 (48.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14 (58.3%)</t>
+          <t>12 (48.0%)</t>
         </is>
       </c>
     </row>
@@ -701,21 +701,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>13 (54.2%)</t>
+          <t>13 (52.0%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (4.2%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10 (41.7%)</t>
+          <t>11 (44.0%)</t>
         </is>
       </c>
     </row>
@@ -747,32 +747,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>7 (36.8%)</t>
+          <t>13 (61.9%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2 (10.5%)</t>
+          <t>1 (4.8%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>7 (33.3%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -780,17 +780,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12 (63.2%)</t>
+          <t>7 (36.8%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1 (5.3%)</t>
+          <t>2 (10.5%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>6 (31.6%)</t>
+          <t>10 (52.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-09
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>91 (52.0%)</t>
+          <t>91 (51.7%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (2.9%)</t>
+          <t>5 (2.8%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>79 (45.1%)</t>
+          <t>80 (45.5%)</t>
         </is>
       </c>
     </row>
@@ -572,32 +572,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10 (33.3%)</t>
+          <t>12 (37.5%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2 (6.7%)</t>
+          <t>2 (6.2%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18 (60.0%)</t>
+          <t>18 (56.2%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -605,7 +605,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12 (40.0%)</t>
+          <t>10 (33.3%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>16 (53.3%)</t>
+          <t>18 (60.0%)</t>
         </is>
       </c>
     </row>
@@ -776,21 +776,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 (36.8%)</t>
+          <t>7 (35.0%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 (10.5%)</t>
+          <t>2 (10.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>11 (55.0%)</t>
         </is>
       </c>
     </row>
@@ -801,11 +801,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>8 (42.1%)</t>
+          <t>9 (45.0%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>11 (57.9%)</t>
+          <t>11 (55.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-12
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>46 (47.4%)</t>
+          <t>47 (48.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6 (6.2%)</t>
+          <t>6 (6.1%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45 (46.4%)</t>
+          <t>45 (45.9%)</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>32 (58.2%)</t>
+          <t>32 (57.1%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>22 (40.0%)</t>
+          <t>23 (41.1%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>26 (49.1%)</t>
+          <t>27 (50.0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>26 (49.1%)</t>
+          <t>26 (48.1%)</t>
         </is>
       </c>
     </row>
@@ -626,53 +626,53 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>18 (66.7%)</t>
+          <t>19 (67.9%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (3.7%)</t>
+          <t>1 (3.6%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8 (29.6%)</t>
+          <t>8 (28.6%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11 (44.0%)</t>
+          <t>12 (46.2%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>2 (7.7%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (56.0%)</t>
+          <t>12 (46.2%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -680,17 +680,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12 (48.0%)</t>
+          <t>11 (44.0%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12 (48.0%)</t>
+          <t>14 (56.0%)</t>
         </is>
       </c>
     </row>
@@ -917,21 +917,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>28 (41.2%)</t>
+          <t>29 (42.0%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5 (7.4%)</t>
+          <t>5 (7.2%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35 (51.5%)</t>
+          <t>35 (50.7%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-13
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -867,11 +867,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100 (50.5%)</t>
+          <t>101 (50.8%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>90 (45.5%)</t>
+          <t>90 (45.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-14
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10 (33.3%)</t>
+          <t>11 (35.5%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (6.7%)</t>
+          <t>2 (6.5%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>18 (60.0%)</t>
+          <t>18 (58.1%)</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -655,42 +655,42 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12 (46.2%)</t>
+          <t>11 (42.3%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2 (7.7%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>12 (46.2%)</t>
+          <t>15 (57.7%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11 (44.0%)</t>
+          <t>12 (46.2%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>2 (7.7%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14 (56.0%)</t>
+          <t>12 (46.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-16
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>91 (51.7%)</t>
+          <t>92 (52.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>80 (45.5%)</t>
+          <t>80 (45.2%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>32 (57.1%)</t>
+          <t>33 (56.9%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (1.8%)</t>
+          <t>1 (1.7%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>23 (41.1%)</t>
+          <t>24 (41.4%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18 (46.2%)</t>
+          <t>18 (45.0%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (15.4%)</t>
+          <t>6 (15.0%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>15 (38.5%)</t>
+          <t>16 (40.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-17
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>47 (48.0%)</t>
+          <t>48 (48.5%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45 (45.9%)</t>
+          <t>45 (45.5%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>18 (45.0%)</t>
+          <t>19 (46.3%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (15.0%)</t>
+          <t>6 (14.6%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16 (40.0%)</t>
+          <t>16 (39.0%)</t>
         </is>
       </c>
     </row>
@@ -772,32 +772,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 (35.0%)</t>
+          <t>10 (47.6%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 (10.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11 (55.0%)</t>
+          <t>11 (52.4%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -805,12 +805,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>9 (45.0%)</t>
+          <t>7 (35.0%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>2 (10.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1017,11 +1017,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21 (51.2%)</t>
+          <t>21 (50.0%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19 (46.3%)</t>
+          <t>20 (47.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-18
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>48 (48.5%)</t>
+          <t>49 (49.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6 (6.1%)</t>
+          <t>6 (6.0%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45 (45.5%)</t>
+          <t>45 (45.0%)</t>
         </is>
       </c>
     </row>
@@ -626,21 +626,21 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>19 (67.9%)</t>
+          <t>20 (69.0%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (3.6%)</t>
+          <t>1 (3.4%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8 (28.6%)</t>
+          <t>8 (27.6%)</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -755,24 +755,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>13 (61.9%)</t>
+          <t>7 (33.3%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1 (4.8%)</t>
+          <t>2 (9.5%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>7 (33.3%)</t>
+          <t>12 (57.1%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -780,42 +780,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>13 (61.9%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.8%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>11 (52.4%)</t>
+          <t>7 (33.3%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>7 (35.0%)</t>
+          <t>10 (47.6%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2 (10.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>11 (55.0%)</t>
+          <t>11 (52.4%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-19
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>92 (52.0%)</t>
+          <t>93 (52.2%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>80 (45.2%)</t>
+          <t>80 (44.9%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>49 (49.0%)</t>
+          <t>49 (48.5%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6 (6.0%)</t>
+          <t>6 (5.9%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>45 (45.0%)</t>
+          <t>46 (45.5%)</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>33 (56.9%)</t>
+          <t>34 (57.6%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>24 (41.4%)</t>
+          <t>24 (40.7%)</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -580,7 +580,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>12 (37.5%)</t>
+          <t>11 (34.4%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -590,32 +590,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18 (56.2%)</t>
+          <t>19 (59.4%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11 (35.5%)</t>
+          <t>12 (37.5%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (6.5%)</t>
+          <t>2 (6.2%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>18 (58.1%)</t>
+          <t>18 (56.2%)</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -730,42 +730,42 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>7 (31.8%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>2 (9.1%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>13 (59.1%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>7 (33.3%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2 (9.5%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12 (57.1%)</t>
+          <t>11 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>75 (48.7%)</t>
+          <t>76 (49.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>72 (46.8%)</t>
+          <t>72 (46.5%)</t>
         </is>
       </c>
     </row>
@@ -1342,21 +1342,21 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>10 (55.6%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1 (5.9%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>6 (35.3%)</t>
+          <t>7 (38.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-20
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>34 (57.6%)</t>
+          <t>35 (58.3%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>24 (40.7%)</t>
+          <t>24 (40.0%)</t>
         </is>
       </c>
     </row>
@@ -526,21 +526,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>27 (50.0%)</t>
+          <t>28 (50.9%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (1.9%)</t>
+          <t>1 (1.8%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>26 (48.1%)</t>
+          <t>26 (47.3%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>19 (46.3%)</t>
+          <t>20 (47.6%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (14.6%)</t>
+          <t>6 (14.3%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16 (39.0%)</t>
+          <t>16 (38.1%)</t>
         </is>
       </c>
     </row>
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11 (34.4%)</t>
+          <t>11 (32.4%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2 (6.2%)</t>
+          <t>3 (8.8%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>19 (59.4%)</t>
+          <t>20 (58.8%)</t>
         </is>
       </c>
     </row>
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11 (42.3%)</t>
+          <t>12 (44.4%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15 (57.7%)</t>
+          <t>15 (55.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-21
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>93 (52.2%)</t>
+          <t>94 (52.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>80 (44.9%)</t>
+          <t>80 (44.7%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-22
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>94 (52.5%)</t>
+          <t>95 (51.9%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (2.8%)</t>
+          <t>5 (2.7%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>80 (44.7%)</t>
+          <t>83 (45.4%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35 (58.3%)</t>
+          <t>36 (58.1%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (1.7%)</t>
+          <t>1 (1.6%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>24 (40.0%)</t>
+          <t>25 (40.3%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>20 (47.6%)</t>
+          <t>21 (48.8%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (14.3%)</t>
+          <t>6 (14.0%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16 (38.1%)</t>
+          <t>16 (37.2%)</t>
         </is>
       </c>
     </row>
@@ -726,21 +726,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>7 (31.8%)</t>
+          <t>7 (30.4%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2 (9.1%)</t>
+          <t>2 (8.7%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13 (59.1%)</t>
+          <t>14 (60.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-23
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>49 (48.5%)</t>
+          <t>49 (48.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>46 (45.5%)</t>
+          <t>47 (46.1%)</t>
         </is>
       </c>
     </row>
@@ -501,11 +501,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>36 (58.1%)</t>
+          <t>37 (57.8%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (40.3%)</t>
+          <t>26 (40.6%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>28 (50.9%)</t>
+          <t>28 (50.0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>26 (47.3%)</t>
+          <t>27 (48.2%)</t>
         </is>
       </c>
     </row>
@@ -776,21 +776,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13 (61.9%)</t>
+          <t>13 (59.1%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1 (4.8%)</t>
+          <t>1 (4.5%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7 (33.3%)</t>
+          <t>8 (36.4%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-24
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>95 (51.9%)</t>
+          <t>95 (51.6%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>83 (45.4%)</t>
+          <t>84 (45.7%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>28 (50.0%)</t>
+          <t>28 (49.1%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>27 (48.2%)</t>
+          <t>28 (49.1%)</t>
         </is>
       </c>
     </row>
@@ -676,21 +676,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12 (46.2%)</t>
+          <t>12 (44.4%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (7.7%)</t>
+          <t>2 (7.4%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12 (46.2%)</t>
+          <t>13 (48.1%)</t>
         </is>
       </c>
     </row>
@@ -1017,21 +1017,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21 (50.0%)</t>
+          <t>21 (48.8%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (2.4%)</t>
+          <t>1 (2.3%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20 (47.6%)</t>
+          <t>21 (48.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-25
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>95 (51.6%)</t>
+          <t>95 (51.4%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>84 (45.7%)</t>
+          <t>85 (45.9%)</t>
         </is>
       </c>
     </row>
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12 (44.4%)</t>
+          <t>12 (42.9%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15 (55.6%)</t>
+          <t>16 (57.1%)</t>
         </is>
       </c>
     </row>
@@ -751,11 +751,11 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>11 (47.8%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>11 (50.0%)</t>
+          <t>12 (52.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-26
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>95 (51.4%)</t>
+          <t>98 (52.1%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>85 (45.9%)</t>
+          <t>85 (45.2%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>49 (48.0%)</t>
+          <t>49 (47.6%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6 (5.9%)</t>
+          <t>6 (5.8%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>47 (46.1%)</t>
+          <t>48 (46.6%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>37 (57.8%)</t>
+          <t>37 (56.9%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (1.6%)</t>
+          <t>2 (3.1%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26 (40.6%)</t>
+          <t>26 (40.0%)</t>
         </is>
       </c>
     </row>
@@ -526,21 +526,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>28 (49.1%)</t>
+          <t>29 (50.0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (1.8%)</t>
+          <t>1 (1.7%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>28 (49.1%)</t>
+          <t>28 (48.3%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21 (48.8%)</t>
+          <t>22 (50.0%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (14.0%)</t>
+          <t>6 (13.6%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16 (37.2%)</t>
+          <t>16 (36.4%)</t>
         </is>
       </c>
     </row>
@@ -676,21 +676,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12 (44.4%)</t>
+          <t>12 (42.9%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (7.4%)</t>
+          <t>2 (7.1%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13 (48.1%)</t>
+          <t>14 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -1192,21 +1192,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13 (59.1%)</t>
+          <t>14 (60.9%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 (9.1%)</t>
+          <t>2 (8.7%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7 (31.8%)</t>
+          <t>7 (30.4%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-27
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11 (32.4%)</t>
+          <t>12 (33.3%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3 (8.8%)</t>
+          <t>3 (8.3%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20 (58.8%)</t>
+          <t>21 (58.3%)</t>
         </is>
       </c>
     </row>
@@ -697,50 +697,50 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Russian Federation</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>13 (52.0%)</t>
+          <t>9 (34.6%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>2 (7.7%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>11 (44.0%)</t>
+          <t>15 (57.7%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Russian Federation</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>7 (30.4%)</t>
+          <t>13 (52.0%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2 (8.7%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14 (60.9%)</t>
+          <t>11 (44.0%)</t>
         </is>
       </c>
     </row>
@@ -801,11 +801,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10 (47.6%)</t>
+          <t>10 (45.5%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -815,7 +815,32 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>11 (52.4%)</t>
+          <t>12 (54.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>5 (33.3%)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1 (6.7%)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>9 (60.0%)</t>
         </is>
       </c>
     </row>
@@ -1317,21 +1342,21 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>11 (55.0%)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2 (10.5%)</t>
+          <t>2 (10.0%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>7 (36.8%)</t>
+          <t>7 (35.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-28
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -917,11 +917,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>76 (49.0%)</t>
+          <t>77 (49.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>72 (46.5%)</t>
+          <t>72 (46.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-29
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>98 (52.1%)</t>
+          <t>98 (51.9%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (2.7%)</t>
+          <t>5 (2.6%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>85 (45.2%)</t>
+          <t>86 (45.5%)</t>
         </is>
       </c>
     </row>
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>12 (33.3%)</t>
+          <t>14 (36.8%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3 (8.3%)</t>
+          <t>3 (7.9%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>21 (58.3%)</t>
+          <t>21 (55.3%)</t>
         </is>
       </c>
     </row>
@@ -651,11 +651,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12 (42.9%)</t>
+          <t>12 (41.4%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -665,7 +665,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>16 (57.1%)</t>
+          <t>17 (58.6%)</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -755,7 +755,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11 (47.8%)</t>
+          <t>10 (43.5%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -765,39 +765,39 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>12 (52.2%)</t>
+          <t>13 (56.5%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13 (59.1%)</t>
+          <t>11 (47.8%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1 (4.5%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>8 (36.4%)</t>
+          <t>12 (52.2%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -805,17 +805,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10 (45.5%)</t>
+          <t>13 (59.1%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.5%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>12 (54.5%)</t>
+          <t>8 (36.4%)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>101 (50.8%)</t>
+          <t>101 (50.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>90 (45.2%)</t>
+          <t>91 (45.5%)</t>
         </is>
       </c>
     </row>
@@ -917,11 +917,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>77 (49.4%)</t>
+          <t>77 (49.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>72 (46.2%)</t>
+          <t>73 (46.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-09-30
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>49 (47.6%)</t>
+          <t>50 (47.6%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6 (5.8%)</t>
+          <t>6 (5.7%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>48 (46.6%)</t>
+          <t>49 (46.7%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12 (37.5%)</t>
+          <t>12 (36.4%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (6.2%)</t>
+          <t>2 (6.1%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>18 (56.2%)</t>
+          <t>19 (57.6%)</t>
         </is>
       </c>
     </row>
@@ -747,40 +747,40 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>10 (43.5%)</t>
+          <t>15 (62.5%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.2%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>13 (56.5%)</t>
+          <t>8 (33.3%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11 (47.8%)</t>
+          <t>11 (45.8%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -790,32 +790,32 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12 (52.2%)</t>
+          <t>13 (54.2%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>13 (59.1%)</t>
+          <t>11 (47.8%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1 (4.5%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>8 (36.4%)</t>
+          <t>12 (52.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-01
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -701,21 +701,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9 (34.6%)</t>
+          <t>9 (33.3%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2 (7.7%)</t>
+          <t>2 (7.4%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>15 (57.7%)</t>
+          <t>16 (59.3%)</t>
         </is>
       </c>
     </row>
@@ -942,21 +942,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>29 (42.0%)</t>
+          <t>30 (42.9%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5 (7.2%)</t>
+          <t>5 (7.1%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35 (50.7%)</t>
+          <t>35 (50.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-14
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>98 (51.9%)</t>
+          <t>104 (50.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (2.6%)</t>
+          <t>7 (3.4%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>86 (45.5%)</t>
+          <t>97 (46.6%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>50 (47.6%)</t>
+          <t>56 (46.3%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6 (5.7%)</t>
+          <t>7 (5.8%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>49 (46.7%)</t>
+          <t>58 (47.9%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>37 (56.9%)</t>
+          <t>39 (56.5%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2 (3.1%)</t>
+          <t>3 (4.3%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26 (40.0%)</t>
+          <t>27 (39.1%)</t>
         </is>
       </c>
     </row>
@@ -526,21 +526,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>29 (50.0%)</t>
+          <t>32 (51.6%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (1.7%)</t>
+          <t>1 (1.6%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>28 (48.3%)</t>
+          <t>29 (46.8%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>22 (50.0%)</t>
+          <t>24 (49.0%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (13.6%)</t>
+          <t>7 (14.3%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>16 (36.4%)</t>
+          <t>18 (36.7%)</t>
         </is>
       </c>
     </row>
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14 (36.8%)</t>
+          <t>14 (35.0%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3 (7.9%)</t>
+          <t>3 (7.5%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>21 (55.3%)</t>
+          <t>23 (57.5%)</t>
         </is>
       </c>
     </row>
@@ -601,121 +601,121 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12 (36.4%)</t>
+          <t>13 (36.1%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (6.1%)</t>
+          <t>2 (5.6%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19 (57.6%)</t>
+          <t>21 (58.3%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20 (69.0%)</t>
+          <t>14 (42.4%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (3.4%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>8 (27.6%)</t>
+          <t>19 (57.6%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12 (41.4%)</t>
+          <t>15 (46.9%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>2 (6.2%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>17 (58.6%)</t>
+          <t>15 (46.9%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12 (42.9%)</t>
+          <t>14 (43.8%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (7.1%)</t>
+          <t>2 (6.2%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14 (50.0%)</t>
+          <t>16 (50.0%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9 (33.3%)</t>
+          <t>20 (66.7%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2 (7.4%)</t>
+          <t>1 (3.3%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>16 (59.3%)</t>
+          <t>9 (30.0%)</t>
         </is>
       </c>
     </row>
@@ -726,71 +726,71 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13 (52.0%)</t>
+          <t>15 (53.6%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>1 (3.6%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11 (44.0%)</t>
+          <t>12 (42.9%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>15 (62.5%)</t>
+          <t>12 (44.4%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1 (4.2%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>8 (33.3%)</t>
+          <t>15 (55.6%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11 (45.8%)</t>
+          <t>15 (60.0%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13 (54.2%)</t>
+          <t>9 (36.0%)</t>
         </is>
       </c>
     </row>
@@ -826,21 +826,21 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>5 (33.3%)</t>
+          <t>6 (37.5%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1 (6.7%)</t>
+          <t>1 (6.2%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>9 (60.0%)</t>
+          <t>9 (56.2%)</t>
         </is>
       </c>
     </row>
@@ -892,21 +892,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>101 (50.5%)</t>
+          <t>103 (50.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8 (4.0%)</t>
+          <t>8 (3.9%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>91 (45.5%)</t>
+          <t>93 (45.6%)</t>
         </is>
       </c>
     </row>
@@ -917,21 +917,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>77 (49.0%)</t>
+          <t>79 (49.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7 (4.5%)</t>
+          <t>7 (4.4%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>73 (46.5%)</t>
+          <t>74 (46.2%)</t>
         </is>
       </c>
     </row>
@@ -942,21 +942,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>30 (42.9%)</t>
+          <t>31 (43.7%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5 (7.1%)</t>
+          <t>5 (7.0%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35 (50.0%)</t>
+          <t>35 (49.3%)</t>
         </is>
       </c>
     </row>
@@ -967,21 +967,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21 (38.2%)</t>
+          <t>22 (37.9%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (5.5%)</t>
+          <t>3 (5.2%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>31 (56.4%)</t>
+          <t>33 (56.9%)</t>
         </is>
       </c>
     </row>
@@ -1092,21 +1092,21 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13 (46.4%)</t>
+          <t>13 (44.8%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1 (3.6%)</t>
+          <t>1 (3.4%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (50.0%)</t>
+          <t>15 (51.7%)</t>
         </is>
       </c>
     </row>
@@ -1117,21 +1117,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14 (50.0%)</t>
+          <t>15 (51.7%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (7.1%)</t>
+          <t>2 (6.9%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12 (42.9%)</t>
+          <t>12 (41.4%)</t>
         </is>
       </c>
     </row>
@@ -1217,21 +1217,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14 (60.9%)</t>
+          <t>15 (62.5%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 (8.7%)</t>
+          <t>2 (8.3%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7 (30.4%)</t>
+          <t>7 (29.2%)</t>
         </is>
       </c>
     </row>
@@ -1363,50 +1363,50 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10 (55.6%)</t>
+          <t>10 (52.6%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>1 (5.3%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7 (38.9%)</t>
+          <t>8 (42.1%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>10 (55.6%)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1 (5.9%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>6 (35.3%)</t>
+          <t>7 (38.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-15
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>104 (50.0%)</t>
+          <t>105 (49.8%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7 (3.4%)</t>
+          <t>7 (3.3%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>97 (46.6%)</t>
+          <t>99 (46.9%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>32 (51.6%)</t>
+          <t>32 (50.8%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>29 (46.8%)</t>
+          <t>30 (47.6%)</t>
         </is>
       </c>
     </row>
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14 (35.0%)</t>
+          <t>14 (34.1%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3 (7.5%)</t>
+          <t>3 (7.3%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>23 (57.5%)</t>
+          <t>24 (58.5%)</t>
         </is>
       </c>
     </row>
@@ -601,21 +601,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13 (36.1%)</t>
+          <t>14 (37.8%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2 (5.6%)</t>
+          <t>2 (5.4%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>21 (58.3%)</t>
+          <t>21 (56.8%)</t>
         </is>
       </c>
     </row>
@@ -626,11 +626,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14 (42.4%)</t>
+          <t>14 (41.2%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>19 (57.6%)</t>
+          <t>20 (58.8%)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>103 (50.5%)</t>
+          <t>104 (50.7%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>93 (45.6%)</t>
+          <t>93 (45.4%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restyle charts for mobile, add CI whiskers, fix n-label offset; fix UTF-8 encoding on Windows
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>82 (53.2%)</t>
+          <t>100 (49.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 (3.2%)</t>
+          <t>7 (3.5%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>67 (43.5%)</t>
+          <t>95 (47.0%)</t>
         </is>
       </c>
     </row>
@@ -476,71 +476,71 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>39 (46.4%)</t>
+          <t>53 (44.9%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5 (6.0%)</t>
+          <t>7 (5.9%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>40 (47.6%)</t>
+          <t>58 (49.2%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>24 (48.0%)</t>
+          <t>35 (55.6%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 (2.0%)</t>
+          <t>3 (4.8%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (50.0%)</t>
+          <t>25 (39.7%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>27 (57.4%)</t>
+          <t>31 (50.0%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1 (2.1%)</t>
+          <t>2 (3.2%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19 (40.4%)</t>
+          <t>29 (46.8%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15 (45.5%)</t>
+          <t>21 (47.7%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5 (15.2%)</t>
+          <t>6 (13.6%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>13 (39.4%)</t>
+          <t>17 (38.6%)</t>
         </is>
       </c>
     </row>
@@ -576,196 +576,196 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10 (33.3%)</t>
+          <t>14 (34.1%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2 (6.7%)</t>
+          <t>3 (7.3%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>18 (60.0%)</t>
+          <t>24 (58.5%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16 (66.7%)</t>
+          <t>13 (39.4%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (4.2%)</t>
+          <t>1 (3.0%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7 (29.2%)</t>
+          <t>19 (57.6%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11 (47.8%)</t>
+          <t>12 (38.7%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (4.3%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11 (47.8%)</t>
+          <t>19 (61.3%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8 (38.1%)</t>
+          <t>12 (40.0%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>2 (6.7%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>13 (61.9%)</t>
+          <t>16 (53.3%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Russian Federation</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10 (50.0%)</t>
+          <t>14 (48.3%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>2 (6.9%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9 (45.0%)</t>
+          <t>13 (44.8%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9 (47.4%)</t>
+          <t>19 (67.9%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (3.6%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>8 (28.6%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Russian Federation</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12 (66.7%)</t>
+          <t>14 (51.9%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>1 (3.7%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>5 (27.8%)</t>
+          <t>12 (44.4%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11 (61.1%)</t>
+          <t>15 (60.0%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1 (5.6%)</t>
+          <t>1 (4.0%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>6 (33.3%)</t>
+          <t>9 (36.0%)</t>
         </is>
       </c>
     </row>
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>7 (41.2%)</t>
+          <t>11 (45.8%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -790,32 +790,32 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>13 (54.2%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>5 (33.3%)</t>
+          <t>10 (45.5%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2 (13.3%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>8 (53.3%)</t>
+          <t>12 (54.5%)</t>
         </is>
       </c>
     </row>
@@ -867,21 +867,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>99 (50.5%)</t>
+          <t>103 (50.7%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8 (4.1%)</t>
+          <t>8 (3.9%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>89 (45.4%)</t>
+          <t>92 (45.3%)</t>
         </is>
       </c>
     </row>
@@ -892,21 +892,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>74 (48.7%)</t>
+          <t>78 (49.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7 (4.6%)</t>
+          <t>7 (4.4%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>71 (46.7%)</t>
+          <t>73 (46.2%)</t>
         </is>
       </c>
     </row>
@@ -917,21 +917,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27 (40.3%)</t>
+          <t>30 (42.9%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5 (7.5%)</t>
+          <t>5 (7.1%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>35 (52.2%)</t>
+          <t>35 (50.0%)</t>
         </is>
       </c>
     </row>
@@ -942,21 +942,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21 (38.2%)</t>
+          <t>22 (37.9%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (5.5%)</t>
+          <t>3 (5.2%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>31 (56.4%)</t>
+          <t>33 (56.9%)</t>
         </is>
       </c>
     </row>
@@ -1017,21 +1017,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21 (51.2%)</t>
+          <t>21 (48.8%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (2.4%)</t>
+          <t>1 (2.3%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19 (46.3%)</t>
+          <t>21 (48.8%)</t>
         </is>
       </c>
     </row>
@@ -1067,21 +1067,21 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13 (46.4%)</t>
+          <t>13 (44.8%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1 (3.6%)</t>
+          <t>1 (3.4%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (50.0%)</t>
+          <t>15 (51.7%)</t>
         </is>
       </c>
     </row>
@@ -1092,21 +1092,21 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14 (50.0%)</t>
+          <t>15 (51.7%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (7.1%)</t>
+          <t>2 (6.9%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12 (42.9%)</t>
+          <t>12 (41.4%)</t>
         </is>
       </c>
     </row>
@@ -1192,21 +1192,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>13 (59.1%)</t>
+          <t>15 (62.5%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2 (9.1%)</t>
+          <t>2 (8.3%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7 (31.8%)</t>
+          <t>7 (29.2%)</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Russian Federation</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1246,24 +1246,24 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14 (70.0%)</t>
+          <t>11 (55.0%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>2 (10.0%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>5 (25.0%)</t>
+          <t>7 (35.0%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1276,27 +1276,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.0%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>6 (30.0%)</t>
+          <t>5 (25.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10 (52.6%)</t>
+          <t>14 (70.0%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1306,14 +1306,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>9 (47.4%)</t>
+          <t>6 (30.0%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Russian Federation</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1326,62 +1326,62 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2 (10.5%)</t>
+          <t>1 (5.3%)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>7 (36.8%)</t>
+          <t>8 (42.1%)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>10 (52.6%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1 (5.9%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>6 (35.3%)</t>
+          <t>9 (47.4%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>10 (55.6%)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1 (5.9%)</t>
+          <t>1 (5.6%)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>6 (35.3%)</t>
+          <t>7 (38.9%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-16
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>53 (44.9%)</t>
+          <t>54 (45.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7 (5.9%)</t>
+          <t>8 (6.7%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>58 (49.2%)</t>
+          <t>58 (48.3%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21 (47.7%)</t>
+          <t>22 (48.9%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (13.6%)</t>
+          <t>6 (13.3%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17 (38.6%)</t>
+          <t>17 (37.8%)</t>
         </is>
       </c>
     </row>
@@ -751,21 +751,21 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>15 (60.0%)</t>
+          <t>15 (57.7%)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1 (4.0%)</t>
+          <t>2 (7.7%)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>9 (36.0%)</t>
+          <t>9 (34.6%)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>78 (49.4%)</t>
+          <t>78 (49.1%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>73 (46.2%)</t>
+          <t>74 (46.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-17
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>54 (45.0%)</t>
+          <t>54 (44.6%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8 (6.7%)</t>
+          <t>8 (6.6%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>58 (48.3%)</t>
+          <t>59 (48.8%)</t>
         </is>
       </c>
     </row>
@@ -1063,32 +1063,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13 (44.8%)</t>
+          <t>15 (48.4%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1 (3.4%)</t>
+          <t>2 (6.5%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15 (51.7%)</t>
+          <t>14 (45.2%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1096,17 +1096,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>13 (44.8%)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1 (3.4%)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>15 (51.7%)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2 (6.9%)</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>12 (41.4%)</t>
         </is>
       </c>
     </row>
@@ -1392,11 +1392,11 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>7 (43.8%)</t>
+          <t>7 (41.2%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>9 (56.2%)</t>
+          <t>10 (58.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-18
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -626,11 +626,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12 (38.7%)</t>
+          <t>13 (40.6%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>19 (61.3%)</t>
+          <t>19 (59.4%)</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -680,42 +680,42 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14 (48.3%)</t>
+          <t>19 (65.5%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2 (6.9%)</t>
+          <t>1 (3.4%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13 (44.8%)</t>
+          <t>9 (31.0%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>19 (67.9%)</t>
+          <t>14 (48.3%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (3.6%)</t>
+          <t>2 (6.9%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>8 (28.6%)</t>
+          <t>13 (44.8%)</t>
         </is>
       </c>
     </row>
@@ -1017,21 +1017,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21 (48.8%)</t>
+          <t>21 (50.0%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (2.3%)</t>
+          <t>1 (2.4%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>21 (48.8%)</t>
+          <t>20 (47.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-19
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,21 +451,21 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100 (49.5%)</t>
+          <t>100 (49.3%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7 (3.5%)</t>
+          <t>7 (3.4%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>95 (47.0%)</t>
+          <t>96 (47.3%)</t>
         </is>
       </c>
     </row>
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>54 (44.6%)</t>
+          <t>54 (44.3%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>59 (48.8%)</t>
+          <t>60 (49.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-20
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -626,11 +626,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13 (40.6%)</t>
+          <t>13 (39.4%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>19 (59.4%)</t>
+          <t>20 (60.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-21
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -1117,21 +1117,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>13 (48.1%)</t>
+          <t>13 (46.4%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1 (3.7%)</t>
+          <t>1 (3.6%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>13 (48.1%)</t>
+          <t>14 (50.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-22
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -867,11 +867,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>103 (50.7%)</t>
+          <t>104 (51.0%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>92 (45.3%)</t>
+          <t>92 (45.1%)</t>
         </is>
       </c>
     </row>
@@ -892,11 +892,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>78 (49.1%)</t>
+          <t>78 (48.8%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>74 (46.5%)</t>
+          <t>75 (46.9%)</t>
         </is>
       </c>
     </row>
@@ -942,21 +942,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>22 (37.9%)</t>
+          <t>22 (37.3%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3 (5.2%)</t>
+          <t>4 (6.8%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>33 (56.9%)</t>
+          <t>33 (55.9%)</t>
         </is>
       </c>
     </row>
@@ -1017,21 +1017,21 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21 (50.0%)</t>
+          <t>22 (51.2%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (2.4%)</t>
+          <t>1 (2.3%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20 (47.6%)</t>
+          <t>20 (46.5%)</t>
         </is>
       </c>
     </row>
@@ -1217,21 +1217,21 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>9 (42.9%)</t>
+          <t>9 (40.9%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1 (4.8%)</t>
+          <t>1 (4.5%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>11 (52.4%)</t>
+          <t>12 (54.5%)</t>
         </is>
       </c>
     </row>
@@ -1242,28 +1242,28 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>11 (55.0%)</t>
+          <t>12 (57.1%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2 (10.0%)</t>
+          <t>2 (9.5%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>7 (35.0%)</t>
+          <t>7 (33.3%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1276,19 +1276,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1 (5.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5 (25.0%)</t>
+          <t>6 (30.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (5.0%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>6 (30.0%)</t>
+          <t>5 (25.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-23
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -967,21 +967,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>26 (48.1%)</t>
+          <t>26 (47.3%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (11.1%)</t>
+          <t>6 (10.9%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>22 (40.7%)</t>
+          <t>23 (41.8%)</t>
         </is>
       </c>
     </row>
@@ -1067,21 +1067,21 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15 (48.4%)</t>
+          <t>15 (46.9%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2 (6.5%)</t>
+          <t>3 (9.4%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14 (45.2%)</t>
+          <t>14 (43.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-24
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100 (49.3%)</t>
+          <t>102 (49.8%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>96 (47.3%)</t>
+          <t>96 (46.8%)</t>
         </is>
       </c>
     </row>
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>54 (44.3%)</t>
+          <t>54 (43.5%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8 (6.6%)</t>
+          <t>9 (7.3%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>60 (49.2%)</t>
+          <t>61 (49.2%)</t>
         </is>
       </c>
     </row>
@@ -597,32 +597,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13 (39.4%)</t>
+          <t>14 (41.2%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (3.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19 (57.6%)</t>
+          <t>20 (58.8%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -635,12 +635,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (3.0%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20 (60.6%)</t>
+          <t>19 (57.6%)</t>
         </is>
       </c>
     </row>
@@ -867,11 +867,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>104 (51.0%)</t>
+          <t>105 (51.2%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>92 (45.1%)</t>
+          <t>92 (44.9%)</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -996,42 +996,42 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>18 (40.9%)</t>
+          <t>23 (52.3%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7 (15.9%)</t>
+          <t>1 (2.3%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>19 (43.2%)</t>
+          <t>20 (45.5%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>22 (51.2%)</t>
+          <t>18 (40.9%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (2.3%)</t>
+          <t>7 (15.9%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20 (46.5%)</t>
+          <t>19 (43.2%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-26
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>102 (49.8%)</t>
+          <t>102 (49.5%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>96 (46.8%)</t>
+          <t>97 (47.1%)</t>
         </is>
       </c>
     </row>
@@ -526,11 +526,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>31 (50.0%)</t>
+          <t>32 (50.8%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>29 (46.8%)</t>
+          <t>29 (46.0%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-27
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -451,11 +451,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>102 (49.5%)</t>
+          <t>102 (49.3%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>97 (47.1%)</t>
+          <t>98 (47.3%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35 (55.6%)</t>
+          <t>35 (54.7%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (4.8%)</t>
+          <t>3 (4.7%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25 (39.7%)</t>
+          <t>26 (40.6%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>22 (48.9%)</t>
+          <t>23 (50.0%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (13.3%)</t>
+          <t>6 (13.0%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17 (37.8%)</t>
+          <t>17 (37.0%)</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -610,37 +610,37 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (2.9%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>20 (58.8%)</t>
+          <t>19 (55.9%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13 (39.4%)</t>
+          <t>14 (41.2%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (3.0%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>19 (57.6%)</t>
+          <t>20 (58.8%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-28
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>54 (43.5%)</t>
+          <t>55 (44.0%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>9 (7.3%)</t>
+          <t>9 (7.2%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>61 (49.2%)</t>
+          <t>61 (48.8%)</t>
         </is>
       </c>
     </row>
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>23 (50.0%)</t>
+          <t>24 (51.1%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (13.0%)</t>
+          <t>6 (12.8%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17 (37.0%)</t>
+          <t>17 (36.2%)</t>
         </is>
       </c>
     </row>
@@ -597,32 +597,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Türkiye</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14 (41.2%)</t>
+          <t>14 (40.0%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1 (2.9%)</t>
+          <t>0 (0.0%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>19 (55.9%)</t>
+          <t>21 (60.0%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Türkiye</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -635,12 +635,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>1 (2.9%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>20 (58.8%)</t>
+          <t>19 (55.9%)</t>
         </is>
       </c>
     </row>
@@ -892,21 +892,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>78 (48.8%)</t>
+          <t>78 (48.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7 (4.4%)</t>
+          <t>8 (5.0%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>75 (46.9%)</t>
+          <t>75 (46.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-29
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,21 +476,21 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>55 (44.0%)</t>
+          <t>55 (43.7%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>9 (7.2%)</t>
+          <t>9 (7.1%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>61 (48.8%)</t>
+          <t>62 (49.2%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35 (54.7%)</t>
+          <t>35 (53.8%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (4.7%)</t>
+          <t>3 (4.6%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26 (40.6%)</t>
+          <t>27 (41.5%)</t>
         </is>
       </c>
     </row>
@@ -526,21 +526,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>32 (50.8%)</t>
+          <t>33 (51.6%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2 (3.2%)</t>
+          <t>2 (3.1%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>29 (46.0%)</t>
+          <t>29 (45.3%)</t>
         </is>
       </c>
     </row>
@@ -776,11 +776,11 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11 (45.8%)</t>
+          <t>11 (44.0%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>13 (54.2%)</t>
+          <t>14 (56.0%)</t>
         </is>
       </c>
     </row>
@@ -1392,11 +1392,11 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>7 (41.2%)</t>
+          <t>8 (44.4%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>10 (58.8%)</t>
+          <t>10 (55.6%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-30
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -551,21 +551,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24 (51.1%)</t>
+          <t>25 (52.1%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 (12.8%)</t>
+          <t>6 (12.5%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>17 (36.2%)</t>
+          <t>17 (35.4%)</t>
         </is>
       </c>
     </row>
@@ -601,11 +601,11 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14 (40.0%)</t>
+          <t>15 (41.7%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>21 (60.0%)</t>
+          <t>21 (58.3%)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh chess stats 2026-10-31
</commit_message>
<xml_diff>
--- a/data/country_outcome_tables.xlsx
+++ b/data/country_outcome_tables.xlsx
@@ -476,11 +476,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>55 (43.7%)</t>
+          <t>56 (44.1%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>62 (49.2%)</t>
+          <t>62 (48.8%)</t>
         </is>
       </c>
     </row>
@@ -501,21 +501,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35 (53.8%)</t>
+          <t>37 (54.4%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3 (4.6%)</t>
+          <t>3 (4.4%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>27 (41.5%)</t>
+          <t>28 (41.2%)</t>
         </is>
       </c>
     </row>
@@ -576,21 +576,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14 (34.1%)</t>
+          <t>14 (33.3%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3 (7.3%)</t>
+          <t>3 (7.1%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>24 (58.5%)</t>
+          <t>25 (59.5%)</t>
         </is>
       </c>
     </row>
@@ -801,11 +801,11 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10 (45.5%)</t>
+          <t>10 (43.5%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>12 (54.5%)</t>
+          <t>13 (56.5%)</t>
         </is>
       </c>
     </row>

</xml_diff>